<commit_message>
Hand Decision Import 2
</commit_message>
<xml_diff>
--- a/data/hand_decision_template.xlsx
+++ b/data/hand_decision_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d33e7414af4da40d/Desktop/Poker/Poker Sites/GG Poker/Studying/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d33e7414af4da40d/Documents/GitHub/PokerDataIngestion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_2843E74F21560A8EA4DD333CDC3B727AC942CA3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{921BBC49-0449-473B-A1DF-DC646271A66F}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_2843E74F21560A8EA4DD333CDC3B727AC942CA3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FF0B8D3-DE00-4074-A242-EC1469750885}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28800" yWindow="780" windowWidth="16200" windowHeight="10125" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="55">
   <si>
     <t>PURPOSE</t>
   </si>
@@ -135,9 +135,6 @@
     <t>notes</t>
   </si>
   <si>
-    <t>SG2595635456</t>
-  </si>
-  <si>
     <t>preflop</t>
   </si>
   <si>
@@ -147,82 +144,61 @@
     <t>JAM</t>
   </si>
   <si>
-    <t>SG2595635302</t>
-  </si>
-  <si>
-    <t>SG2595635131</t>
-  </si>
-  <si>
-    <t>SG2595634936</t>
-  </si>
-  <si>
-    <t>SG2595634781</t>
-  </si>
-  <si>
-    <t>SG2595634621</t>
-  </si>
-  <si>
-    <t>SG2595634557</t>
-  </si>
-  <si>
-    <t>SG2595634451</t>
-  </si>
-  <si>
-    <t>SG2595634254</t>
-  </si>
-  <si>
-    <t>SG2595634135</t>
-  </si>
-  <si>
-    <t>SG2595633850</t>
-  </si>
-  <si>
-    <t>SG2595633768</t>
-  </si>
-  <si>
     <t>CALL</t>
-  </si>
-  <si>
-    <t>97o at 15bb 3H SB - Facing 3.5x raise from BTN</t>
   </si>
   <si>
     <t>CHECK</t>
   </si>
   <si>
-    <t>A4o at 14bb 3H BTN - Min Raise was correct but then should have folded to AI and call</t>
-  </si>
-  <si>
     <t>RAISE</t>
   </si>
   <si>
-    <t>K9o at 21bb HU BB - Should have been 3x raise</t>
+    <t>SG2475659007</t>
   </si>
   <si>
-    <t>87o at 15bb HU SB - It is 51/49 raise</t>
+    <t>99 15bb 3H SB - Facing 3x raise from BTN</t>
   </si>
   <si>
-    <t>Q6o 12bb HU BB - SB limped</t>
+    <t>SG2482037285</t>
   </si>
   <si>
-    <t>84o 13bb HU SB - Limp all offsuit 4s</t>
+    <t>Q5s 15bb 3H BB - Solver has 2x raise as call, reality - BTN made it 3x</t>
   </si>
   <si>
-    <t>AJo 12bb HU BB - Jam A2o through AJo</t>
+    <t>SG2482037637</t>
   </si>
   <si>
-    <t>J4o 10bb HU SB - Limp 54o through K4o except 94o</t>
+    <t>A5o 12bb 3H SB - BTN fold, Jam A2o through AKo</t>
   </si>
   <si>
-    <t>93o 8bb HU SB - Check all offsuit 9s when limped</t>
+    <t>SG2482037803</t>
   </si>
   <si>
-    <t>Q2s 9bb HU SB - Jam Q4s through Q7s, limp all other suited Queens</t>
+    <t>72o 13bb 3H BTN - Fold all offsuit 2s</t>
   </si>
   <si>
-    <t>74o 4bb HU SB - No solution for this but check weak hands when limped</t>
+    <t>SG2482037992</t>
   </si>
   <si>
-    <t>K8o 3bb HU SB - Jam all offsuit Kings &lt;=9 bbs</t>
+    <t>Q3o 11bb 3H BB - Should be a 3x raise - raising some offsuit Q at this stack depth</t>
+  </si>
+  <si>
+    <t>SG2482038381</t>
+  </si>
+  <si>
+    <t>99 9bb 3H SB - Correct raise sizing of 2.5x, 22 through 88 is jam</t>
+  </si>
+  <si>
+    <t>SG2482038527</t>
+  </si>
+  <si>
+    <t>54s 10bb 3H BTN - Fold 54s through Q4s</t>
+  </si>
+  <si>
+    <t>SG2482038692</t>
+  </si>
+  <si>
+    <t>99 10bb 3H BB - Jam vs BTN Raise. Only calling AA, all other pairs are jams</t>
   </si>
 </sst>
 </file>
@@ -800,265 +776,210 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="C2" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2" s="5" t="b">
-        <f t="shared" ref="E2" si="0">IF(C2="","",IF(D2="","",C2=D2))</f>
+        <f t="shared" ref="E2:E9" si="0">IF(C2="","",IF(D2="","",C2=D2))</f>
         <v>1</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="E3" s="5" t="b">
-        <f t="shared" ref="E3:E66" si="1">IF(C3="","",IF(D3="","",C3=D3))</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="E4" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E5" s="5" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>35</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E8" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E9" s="5" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>51</v>
-      </c>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="5" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>49</v>
-      </c>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="E14" s="5"/>
       <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1067,7 +988,7 @@
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E3:E66" si="1">IF(C15="","",IF(D15="","",C15=D15))</f>
         <v/>
       </c>
       <c r="F15" s="6"/>
@@ -5863,7 +5784,7 @@
       <c r="C451" s="4"/>
       <c r="D451" s="4"/>
       <c r="E451" s="5" t="str">
-        <f t="shared" ref="E451:E514" si="8">IF(C451="","",IF(D451="","",C451=D451))</f>
+        <f t="shared" ref="E451:E502" si="8">IF(C451="","",IF(D451="","",C451=D451))</f>
         <v/>
       </c>
       <c r="F451" s="6"/>

</xml_diff>

<commit_message>
Updated hand decision template 3
</commit_message>
<xml_diff>
--- a/data/hand_decision_template.xlsx
+++ b/data/hand_decision_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d33e7414af4da40d/Documents/GitHub/PokerDataIngestion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="11_2843E74F21560A8EA4DD333CDC3B727AC942CA3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FF0B8D3-DE00-4074-A242-EC1469750885}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="11_2843E74F21560A8EA4DD333CDC3B727AC942CA3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{450F544B-5BE7-4AED-92B8-A3407A7503F3}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="780" windowWidth="16200" windowHeight="10125" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>PURPOSE</t>
   </si>
@@ -147,58 +147,28 @@
     <t>CALL</t>
   </si>
   <si>
-    <t>CHECK</t>
+    <t>SG2664720855</t>
   </si>
   <si>
-    <t>RAISE</t>
+    <t>KJo 15bb 3H BB - Only call KQo, AJo+</t>
   </si>
   <si>
-    <t>SG2475659007</t>
+    <t>SG2664721158</t>
   </si>
   <si>
-    <t>99 15bb 3H SB - Facing 3x raise from BTN</t>
+    <t>K7s 14bb HU SB - Limp called 3x raise by BB. Limp-call all suited K</t>
   </si>
   <si>
-    <t>SG2482037285</t>
+    <t>SG2664721465</t>
   </si>
   <si>
-    <t>Q5s 15bb 3H BB - Solver has 2x raise as call, reality - BTN made it 3x</t>
+    <t>JJ 19bb HU BB - Call all pairs and A3s+</t>
   </si>
   <si>
-    <t>SG2482037637</t>
+    <t>SG2664721633</t>
   </si>
   <si>
-    <t>A5o 12bb 3H SB - BTN fold, Jam A2o through AKo</t>
-  </si>
-  <si>
-    <t>SG2482037803</t>
-  </si>
-  <si>
-    <t>72o 13bb 3H BTN - Fold all offsuit 2s</t>
-  </si>
-  <si>
-    <t>SG2482037992</t>
-  </si>
-  <si>
-    <t>Q3o 11bb 3H BB - Should be a 3x raise - raising some offsuit Q at this stack depth</t>
-  </si>
-  <si>
-    <t>SG2482038381</t>
-  </si>
-  <si>
-    <t>99 9bb 3H SB - Correct raise sizing of 2.5x, 22 through 88 is jam</t>
-  </si>
-  <si>
-    <t>SG2482038527</t>
-  </si>
-  <si>
-    <t>54s 10bb 3H BTN - Fold 54s through Q4s</t>
-  </si>
-  <si>
-    <t>SG2482038692</t>
-  </si>
-  <si>
-    <t>99 10bb 3H BB - Jam vs BTN Raise. Only calling AA, all other pairs are jams</t>
+    <t>Q4s 6bb HU SB - Jam Q2s+ through AKs</t>
   </si>
 </sst>
 </file>
@@ -315,6 +285,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -776,178 +750,141 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="5" t="b">
-        <f t="shared" ref="E2:E9" si="0">IF(C2="","",IF(D2="","",C2=D2))</f>
+        <f t="shared" ref="E2:E16" si="0">IF(C2="","",IF(D2="","",C2=D2))</f>
         <v>1</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E3" s="5" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E4" s="5" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5" s="5" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="5" t="b">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>48</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="5" t="b">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>50</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="5" t="b">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>52</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="5" t="b">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>54</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -955,7 +892,10 @@
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
-      <c r="E11" s="5"/>
+      <c r="E11" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -963,7 +903,10 @@
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -971,7 +914,10 @@
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -979,7 +925,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
+      <c r="E14" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -988,7 +937,7 @@
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="5" t="str">
-        <f t="shared" ref="E3:E66" si="1">IF(C15="","",IF(D15="","",C15=D15))</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F15" s="6"/>
@@ -999,7 +948,7 @@
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F16" s="6"/>
@@ -1010,7 +959,7 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E15:E66" si="1">IF(C17="","",IF(D17="","",C17=D17))</f>
         <v/>
       </c>
       <c r="F17" s="6"/>

</xml_diff>

<commit_message>
Hand Decision Template Update
</commit_message>
<xml_diff>
--- a/data/hand_decision_template.xlsx
+++ b/data/hand_decision_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d33e7414af4da40d/Documents/GitHub/PokerDataIngestion/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwent\OneDrive\Documents\GitHub\PokerDataIngestion\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="11_2843E74F21560A8EA4DD333CDC3B727AC942CA3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{450F544B-5BE7-4AED-92B8-A3407A7503F3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81162E9-C4CC-47FE-B87F-F1C4620EDEEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6495" yWindow="3225" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="55">
   <si>
     <t>PURPOSE</t>
   </si>
@@ -147,28 +147,58 @@
     <t>CALL</t>
   </si>
   <si>
-    <t>SG2664720855</t>
+    <t>SG3685605802</t>
   </si>
   <si>
-    <t>KJo 15bb 3H BB - Only call KQo, AJo+</t>
+    <t>SG3685606001</t>
   </si>
   <si>
-    <t>SG2664721158</t>
+    <t>RAISE</t>
   </si>
   <si>
-    <t>K7s 14bb HU SB - Limp called 3x raise by BB. Limp-call all suited K</t>
+    <t>SG3685606214</t>
   </si>
   <si>
-    <t>SG2664721465</t>
+    <t>Q4o 15bb 3H BTN - Fold Q9o and below. Minraise QT/QJo</t>
   </si>
   <si>
-    <t>JJ 19bb HU BB - Call all pairs and A3s+</t>
+    <t>SG3685606293</t>
   </si>
   <si>
-    <t>SG2664721633</t>
+    <t>CHECK</t>
   </si>
   <si>
-    <t>Q4s 6bb HU SB - Jam Q2s+ through AKs</t>
+    <t>94o 15bb 3H BB - 92o - 94o is check, 95/96o is 3x raise when SB limps</t>
+  </si>
+  <si>
+    <t>SG3685606674</t>
+  </si>
+  <si>
+    <t>SG3685607137</t>
+  </si>
+  <si>
+    <t>SG3685607307</t>
+  </si>
+  <si>
+    <t>KQo 13bb 3H SB - 50/50 mix between call and raise. Treated BTN limp as fold</t>
+  </si>
+  <si>
+    <t>98o 10bb 3H BTN - Minraise K9o, Jam JT/QJ/KTo+ all AXo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A7o 13bb 3H SB - Since BTN limped, I treated as fold. Jam all AXo when folded to </t>
+  </si>
+  <si>
+    <t>KJo 15bb 3H BB - Jam K2o and AXo, call all other offsuit K</t>
+  </si>
+  <si>
+    <t>SG3685607633</t>
+  </si>
+  <si>
+    <t>KQo 10bb 3H BB - Call KTo+, A3o+, QJo</t>
+  </si>
+  <si>
+    <t>K5s 1.5bb 3H BTN - Allin with all hands</t>
   </si>
 </sst>
 </file>
@@ -285,10 +315,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -756,73 +782,73 @@
         <v>33</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E2" s="5" t="b">
         <f t="shared" ref="E2:E16" si="0">IF(C2="","",IF(D2="","",C2=D2))</f>
         <v>1</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="5" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E4" s="5" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E5" s="5" t="b">
         <f t="shared" si="0"/>
@@ -833,48 +859,88 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5" t="str">
+      <c r="A6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="5" t="b">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F6" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5" t="str">
+      <c r="A7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="5" t="b">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F7" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="5" t="str">
+      <c r="A8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="5" t="b">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F8" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5" t="str">
+      <c r="A9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="5" t="b">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F9" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
@@ -959,7 +1025,7 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="5" t="str">
-        <f t="shared" ref="E15:E66" si="1">IF(C17="","",IF(D17="","",C17=D17))</f>
+        <f t="shared" ref="E17:E66" si="1">IF(C17="","",IF(D17="","",C17=D17))</f>
         <v/>
       </c>
       <c r="F17" s="6"/>

</xml_diff>